<commit_message>
feat: integrate chat interface and output viewer
- Add Chat & Skill Runner UI with live preview support
- Update navigation bar with new action buttons and responsiveness
- Include pre-compiled file tree for offline browsing
- Add helper for automated versioning and output path management
</commit_message>
<xml_diff>
--- a/skills/jira-import/templates/ISC_FTI-SAL_v3.1 Sprint 2_Project Plan_v1.0.xlsx
+++ b/skills/jira-import/templates/ISC_FTI-SAL_v3.1 Sprint 2_Project Plan_v1.0.xlsx
@@ -112,166 +112,145 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="364">
   <si>
-    <t xml:space="preserve">PROJECT PLANNING</t>
+    <t>PROJECT PLANNING</t>
   </si>
   <si>
-    <t xml:space="preserve">Mã hiệu</t>
+    <t>Mã hiệu</t>
   </si>
   <si>
-    <t xml:space="preserve">3.0-BM/PM/HDCV/FTEL</t>
+    <t>3.0-BM/PM/HDCV/FTEL</t>
   </si>
   <si>
-    <t xml:space="preserve">Phiên bản</t>
+    <t>Phiên bản</t>
   </si>
   <si>
-    <t xml:space="preserve">3/0</t>
+    <t>3/0</t>
   </si>
   <si>
-    <t xml:space="preserve">Hướng dẫn sử dụng Template Project Plan</t>
+    <t>Hướng dẫn sử dụng Template Project Plan</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Phạm vi áp dụng</t>
+    <t>1. Phạm vi áp dụng</t>
   </si>
   <si>
-    <t xml:space="preserve">• Áp dụng cho các dự án mới hoặc nâng cấp có Impact từ Medium trở lên (Medium/High).</t>
+    <t>• Áp dụng cho các dự án mới hoặc nâng cấp có Impact từ Medium trở lên (Medium/High).</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Cấu trúc file (các sheet trong template)</t>
+    <t>2. Cấu trúc file (các sheet trong template)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Cover: Trang bìa, thể hiện mã hiệu tài liệu, phiên bản.</t>
+    <t>• Cover: Trang bìa, thể hiện mã hiệu tài liệu, phiên bản.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Plan: Kế hoạch công việc chi tiết (WBS) theo Module/Main task → Task.</t>
+    <t>• Plan: Kế hoạch công việc chi tiết (WBS) theo Module/Main task → Task.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Guideline: Hướng dẫn sử dụng template (chính là sheet này).</t>
+    <t>• Guideline: Hướng dẫn sử dụng template (chính là sheet này).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Org Chart &amp; Communication (opt - không bắt buộc ): Sơ đồ tổ chức dự án và kế hoạch giao tiếp.</t>
+    <t>• Org Chart &amp; Communication (opt - không bắt buộc ): Sơ đồ tổ chức dự án và kế hoạch giao tiếp.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Objective (opt - không bắt buộc ): Mục tiêu dự án theo các chỉ số PCV, CSAT, SPI, CPI.</t>
+    <t>• Objective (opt - không bắt buộc ): Mục tiêu dự án theo các chỉ số PCV, CSAT, SPI, CPI.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lưu ý:</t>
+    <t>Lưu ý:</t>
   </si>
   <si>
-    <t xml:space="preserve">• Khi triển khai dự án, PM chọn “Make a copy Template Project Plan” để dùng riêng cho dự án.</t>
+    <t>• Khi triển khai dự án, PM chọn “Make a copy Template Project Plan” để dùng riêng cho dự án.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ở bản copy cho dự án, có thể hide hoặc xóa các sheet “(opt -  không bắt buộc)” nếu không dùng.</t>
+    <t>• Ở bản copy cho dự án, có thể hide hoặc xóa các sheet “(opt -  không bắt buộc)” nếu không dùng.</t>
   </si>
   <si>
     <t xml:space="preserve">• Các sheet “(opt)” được khuyến khích sử dụng cho dự án có mức độ phức tạp High để nâng cao chất lượng quản lý, </t>
   </si>
   <si>
-    <t xml:space="preserve">nhưng không bắt buộc áp dụng cho 100% dự án.</t>
+    <t>nhưng không bắt buộc áp dụng cho 100% dự án.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Cách sử dụng</t>
+    <t>3. Cách sử dụng</t>
   </si>
   <si>
-    <t xml:space="preserve">Bước 1 – Khởi tạo file</t>
+    <t>Bước 1 – Khởi tạo file</t>
   </si>
   <si>
-    <t xml:space="preserve">Bước 2 – Lập kế hoạch chi tiết (sheet Plan)</t>
+    <t>Bước 2 – Lập kế hoạch chi tiết (sheet Plan)</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Cập nhật và Lưu trữ</t>
+    <t>4. Cập nhật và Lưu trữ</t>
   </si>
   <si>
-    <t xml:space="preserve">4.1 Trong quá trình triển khai:</t>
+    <t>4.1 Trong quá trình triển khai:</t>
   </si>
   <si>
-    <t xml:space="preserve">• PM cập nhật sheet Plan tối thiểu mỗi tuần hoặc mỗi sprint review.</t>
+    <t>• PM cập nhật sheet Plan tối thiểu mỗi tuần hoặc mỗi sprint review.</t>
   </si>
   <si>
-    <t xml:space="preserve">4.2 Sau khi kết thúc dự án:</t>
+    <t>4.2 Sau khi kết thúc dự án:</t>
   </si>
   <si>
-    <t xml:space="preserve">• Chốt % Done, note rõ các task chưa hoàn thành và lý do.</t>
+    <t>• Chốt % Done, note rõ các task chưa hoàn thành và lý do.</t>
   </si>
   <si>
-    <t xml:space="preserve">• QA/PIC lưu trữ vào tài liệu vào Thư mục dự án.</t>
+    <t>• QA/PIC lưu trữ vào tài liệu vào Thư mục dự án.</t>
   </si>
   <si>
-    <t xml:space="preserve">- **4.1 Trong quá trình triển khai dự án**</t>
+    <t>- **4.1 Trong quá trình triển khai dự án**</t>
   </si>
   <si>
-    <t xml:space="preserve">- PM cập nhật sheet **Plan** &amp; **RADI/Risk** tối thiểu **mỗi tuần hoặc mỗi sprint review**.</t>
+    <t>- PM cập nhật sheet **Plan** &amp; **RADI/Risk** tối thiểu **mỗi tuần hoặc mỗi sprint review**.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Thay đổi phạm vi lớn (scope/impact) cần được phản ánh vào:</t>
+    <t>- Thay đổi phạm vi lớn (scope/impact) cần được phản ánh vào:</t>
   </si>
   <si>
-    <t xml:space="preserve">- Plan (thêm/bớt task, điều chỉnh timeline/effort)</t>
+    <t>- Plan (thêm/bớt task, điều chỉnh timeline/effort)</t>
   </si>
   <si>
-    <t xml:space="preserve">- Risk (thêm risk mới nếu có)</t>
+    <t>- Risk (thêm risk mới nếu có)</t>
   </si>
   <si>
-    <t xml:space="preserve">- Objective (cập nhật lại target nếu đã được PO/Stakeholder thống nhất)</t>
+    <t>- Objective (cập nhật lại target nếu đã được PO/Stakeholder thống nhất)</t>
   </si>
   <si>
-    <t xml:space="preserve">- **4.2 Sau khi kết thúc dự án**</t>
+    <t>- **4.2 Sau khi kết thúc dự án**</t>
   </si>
   <si>
-    <t xml:space="preserve">- PM chốt:</t>
+    <t>- PM chốt:</t>
   </si>
   <si>
-    <t xml:space="preserve">- % Done = 100% cho các task hoàn thành, note lại các task chưa làm và lý do.</t>
+    <t>- % Done = 100% cho các task hoàn thành, note lại các task chưa làm và lý do.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Risk status (Closed / Accepted / Transfered).</t>
+    <t>- Risk status (Closed / Accepted / Transfered).</t>
   </si>
   <si>
-    <t xml:space="preserve">- File Project Plan (bản cuối cùng) được:</t>
+    <t>- File Project Plan (bản cuối cùng) được:</t>
   </si>
   <si>
-    <t xml:space="preserve">- Lưu tại **Fproject** / thư mục share chính thức của dự án.</t>
+    <t>- Lưu tại **Fproject** / thư mục share chính thức của dự án.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Link đính kèm trong **Project Closing / Release Note** theo quy định SQA/ISO.</t>
+    <t>- Link đính kèm trong **Project Closing / Release Note** theo quy định SQA/ISO.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Không chỉnh sửa bản **template master**; mọi cải tiến template phải thông qua đầu mối SQA/PMO ISC.</t>
+    <t>- Không chỉnh sửa bản **template master**; mọi cải tiến template phải thông qua đầu mối SQA/PMO ISC.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="23"/>
-        <color rgb="FFED7D31"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[FTI-SAL v3.1 Sprint 2]</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="23"/>
-        <color rgb="FF0B5394"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Project Planning ➜</t>
-    </r>
+    <t>[FTI-SAL v3.1 Sprint 2] Project Planning ➜</t>
   </si>
   <si>
-    <t xml:space="preserve">Goal</t>
+    <t>Goal</t>
   </si>
   <si>
-    <t xml:space="preserve">Hoàn thiện toàn bộ phân hệ tính lương và phân bổ hóa đơn trả trước Cloudhub, tích hợp tự động Inside-SAL, mở rộng danh mục FOXSG, nâng cấp Core lương và tối ưu hóa quy trình nghiệp vụ cho Kế toán (AF) và Trưởng đơn vị (TDV) với sự hỗ trợ từ AI Code Assistant (Rút ngắn thời gian phát triển xuống 6 tuần).</t>
+    <t>Hoàn thiện toàn bộ phân hệ tính lương và phân bổ hóa đơn trả trước Cloudhub, tích hợp tự động Inside-SAL, mở rộng danh mục FOXSG, nâng cấp Core lương và tối ưu hóa quy trình nghiệp vụ cho Kế toán (AF) và Trưởng đơn vị (TDV) với sự hỗ trợ từ AI Code Assistant (Rút ngắn thời gian phát triển xuống 6 tuần).</t>
   </si>
   <si>
-    <t xml:space="preserve">Start Date</t>
+    <t>Start Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Output/ Module</t>
+    <t>Output/ Module</t>
   </si>
   <si>
     <t xml:space="preserve">Tính được lương Cloudhub trên hệ thống lương cho trường hợp bình thường và các trường hợp đặc thù
@@ -279,10 +258,10 @@
 Trường hợp của các hợp đồng đại diện (sử dụng hợp đồng đại diện để xuất hoá đơn, hợp đồng để tính lương cho kinh doanh là 1 hợp đồng khác) </t>
   </si>
   <si>
-    <t xml:space="preserve">Due Date</t>
+    <t>Due Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Description</t>
+    <t>Description</t>
   </si>
   <si>
     <t xml:space="preserve">1. Sprint Timeline: 17/08/2026 – 07/10/2026
@@ -294,588 +273,588 @@
 9. Sprint Staging Release: 07/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Effort</t>
+    <t>Total Effort</t>
   </si>
   <si>
-    <t xml:space="preserve">PROJECT DETAILS</t>
+    <t>PROJECT DETAILS</t>
   </si>
   <si>
     <t xml:space="preserve">MODULE/ 
 MAIN TASK</t>
   </si>
   <si>
-    <t xml:space="preserve">TASK NAME</t>
+    <t>TASK NAME</t>
   </si>
   <si>
-    <t xml:space="preserve">DESCRIPTION</t>
+    <t>DESCRIPTION</t>
   </si>
   <si>
-    <t xml:space="preserve">PIC</t>
+    <t>PIC</t>
   </si>
   <si>
-    <t xml:space="preserve">% DONE</t>
+    <t>% DONE</t>
   </si>
   <si>
-    <t xml:space="preserve">START DATE</t>
+    <t>START DATE</t>
   </si>
   <si>
-    <t xml:space="preserve">DUE DATE</t>
+    <t>DUE DATE</t>
   </si>
   <si>
     <t xml:space="preserve">EFFORT 
 (Hour)</t>
   </si>
   <si>
-    <t xml:space="preserve">NOTE</t>
+    <t>NOTE</t>
   </si>
   <si>
-    <t xml:space="preserve">EPIC-0. Init Sprint - Kick-off, Analysis &amp; Setup</t>
+    <t>EPIC-0. Init Sprint - Kick-off, Analysis &amp; Setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Project Management</t>
+    <t>Project Management</t>
   </si>
   <si>
-    <t xml:space="preserve">Tổ chức Sprint Planning &amp; Kick-off Sprint 2 (Mô hình AI-assisted)</t>
+    <t>Tổ chức Sprint Planning &amp; Kick-off Sprint 2 (Mô hình AI-assisted)</t>
   </si>
   <si>
-    <t xml:space="preserve">Khởi động Sprint 2, lập kế hoạch và thiết lập Risk Register.</t>
+    <t>Khởi động Sprint 2, lập kế hoạch và thiết lập Risk Register.</t>
   </si>
   <si>
-    <t xml:space="preserve">DuyVM4</t>
+    <t>DuyVM4</t>
   </si>
   <si>
-    <t xml:space="preserve">Thống nhất 19 hạng mục, timeline 6 tuần, mô hình AI-assisted.</t>
+    <t>Thống nhất 19 hạng mục, timeline 6 tuần, mô hình AI-assisted.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lập kế hoạch quản lý tiến độ &amp; Risk Register Sprint 2</t>
+    <t>Lập kế hoạch quản lý tiến độ &amp; Risk Register Sprint 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Kiểm soát rủi ro chất lượng code AI và giải thuật Core lương.</t>
+    <t>Kiểm soát rủi ro chất lượng code AI và giải thuật Core lương.</t>
   </si>
   <si>
-    <t xml:space="preserve">Theo dõi tiến độ &amp; điều phối công việc Tuần</t>
+    <t>Theo dõi tiến độ &amp; điều phối công việc Tuần</t>
   </si>
   <si>
-    <t xml:space="preserve">Giám sát tiến độ tuần, đảm bảo đúng milestone URD &amp; Tech design.</t>
+    <t>Giám sát tiến độ tuần, đảm bảo đúng milestone URD &amp; Tech design.</t>
   </si>
   <si>
-    <t xml:space="preserve">Check task QC &amp; điều phối</t>
+    <t>Check task QC &amp; điều phối</t>
   </si>
   <si>
-    <t xml:space="preserve">Kiểm soát tiến độ bàn giao và chuẩn bị testcase QC.</t>
+    <t>Kiểm soát tiến độ bàn giao và chuẩn bị testcase QC.</t>
   </si>
   <si>
-    <t xml:space="preserve">Requirement &amp; Analysis</t>
+    <t>Requirement &amp; Analysis</t>
   </si>
   <si>
-    <t xml:space="preserve">Phân tích yêu cầu nghiệp vụ 10 tính năng mới</t>
+    <t>Phân tích yêu cầu nghiệp vụ 10 tính năng mới</t>
   </si>
   <si>
-    <t xml:space="preserve">Phân tích nghiệp vụ 19 hạng mục và hoàn tất URD.</t>
+    <t>Phân tích nghiệp vụ 19 hạng mục và hoàn tất URD.</t>
   </si>
   <si>
-    <t xml:space="preserve">NgocDH18</t>
+    <t>NgocDH18</t>
   </si>
   <si>
-    <t xml:space="preserve">Làm rõ luồng phân bổ AF, phân tách TDV, API Inside, bảng lương.</t>
+    <t>Làm rõ luồng phân bổ AF, phân tách TDV, API Inside, bảng lương.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phân tích yêu cầu 5 hạng mục nâng cấp &amp; điều chỉnh</t>
+    <t>Phân tích yêu cầu 5 hạng mục nâng cấp &amp; điều chỉnh</t>
   </si>
   <si>
-    <t xml:space="preserve">Làm rõ khác biệt giữa luồng trả tháng v2.3 và trả trước.</t>
+    <t>Làm rõ khác biệt giữa luồng trả tháng v2.3 và trả trước.</t>
   </si>
   <si>
-    <t xml:space="preserve">Thiết kế Wireframe &amp; UI Mockup các màn hình mới và cập nhật</t>
+    <t>Thiết kế Wireframe &amp; UI Mockup các màn hình mới và cập nhật</t>
   </si>
   <si>
-    <t xml:space="preserve">UI phân bổ AF, phân tách TDV, form sửa lương TDV, tab bảng lương trả trước, danh mục FOXSG</t>
+    <t>UI phân bổ AF, phân tách TDV, form sửa lương TDV, tab bảng lương trả trước, danh mục FOXSG</t>
   </si>
   <si>
-    <t xml:space="preserve">Viết PRD tổng thể và lấy Sign-off từ Stakeholder</t>
+    <t>Viết PRD tổng thể và lấy Sign-off từ Stakeholder</t>
   </si>
   <si>
-    <t xml:space="preserve">Hoàn tất URD đầy đủ trong W1, là điều kiện tiên quyết cho QC Onboarding và DEV implement</t>
+    <t>Hoàn tất URD đầy đủ trong W1, là điều kiện tiên quyết cho QC Onboarding và DEV implement</t>
   </si>
   <si>
-    <t xml:space="preserve">Architecture &amp; Database</t>
+    <t>Architecture &amp; Database</t>
   </si>
   <si>
-    <t xml:space="preserve">Review kiến trúc Core lương v2.3 &amp; thiết lập môi trường Dev (AI-supported)</t>
+    <t>Review kiến trúc Core lương v2.3 &amp; thiết lập môi trường Dev (AI-supported)</t>
   </si>
   <si>
-    <t xml:space="preserve">Khảo sát kiến trúc hiện tại và thiết kế DB hóa đơn trả trước.</t>
+    <t>Khảo sát kiến trúc hiện tại và thiết kế DB hóa đơn trả trước.</t>
   </si>
   <si>
-    <t xml:space="preserve">SonNH103</t>
+    <t>SonNH103</t>
   </si>
   <si>
-    <t xml:space="preserve">Đánh giá khả năng mở rộng Core tính lương và cấu hình AI Assistant cho project</t>
+    <t>Đánh giá khả năng mở rộng Core tính lương và cấu hình AI Assistant cho project</t>
   </si>
   <si>
-    <t xml:space="preserve">Thiết kế Database cho dữ liệu hóa đơn trả trước và quan hệ bảng</t>
+    <t>Thiết kế Database cho dữ liệu hóa đơn trả trước và quan hệ bảng</t>
   </si>
   <si>
-    <t xml:space="preserve">Thiết kế các bảng lưu trữ hóa đơn trả trước, bảng phân bổ AF, phân tách TDV, khóa ngoại và quan hệ</t>
+    <t>Thiết kế các bảng lưu trữ hóa đơn trả trước, bảng phân bổ AF, phân tách TDV, khóa ngoại và quan hệ</t>
   </si>
   <si>
-    <t xml:space="preserve">Tạo DB Migration script và thiết lập dữ liệu mẫu môi trường Dev</t>
+    <t>Tạo DB Migration script và thiết lập dữ liệu mẫu môi trường Dev</t>
   </si>
   <si>
-    <t xml:space="preserve">Chạy migration trên DB Dev, verify index tối ưu hiệu năng cho truy vấn lớn</t>
+    <t>Chạy migration trên DB Dev, verify index tối ưu hiệu năng cho truy vấn lớn</t>
   </si>
   <si>
-    <t xml:space="preserve">EPIC-1. Quản lý phân bổ và giá vốn cho Kế toán (AF)</t>
+    <t>EPIC-1. Quản lý phân bổ và giá vốn cho Kế toán (AF)</t>
   </si>
   <si>
-    <t xml:space="preserve">Kế toán - Phân bổ</t>
+    <t>Kế toán - Phân bổ</t>
   </si>
   <si>
-    <t xml:space="preserve">Xây dựng Backend API khởi tạo dữ liệu phân bổ gốc cho kế toán (AI-assisted)</t>
+    <t>Xây dựng Backend API khởi tạo dữ liệu phân bổ gốc cho kế toán (AI-assisted)</t>
   </si>
   <si>
-    <t xml:space="preserve">Khởi tạo và cấu hình dữ liệu phân bổ gốc cho Kế toán (AF).</t>
+    <t>Khởi tạo và cấu hình dữ liệu phân bổ gốc cho Kế toán (AF).</t>
   </si>
   <si>
-    <t xml:space="preserve">API validate kỳ lương, tỷ lệ và giá trị phân bổ ban đầu.</t>
+    <t>API validate kỳ lương, tỷ lệ và giá trị phân bổ ban đầu.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phát triển giao diện màn hình khởi tạo phân bổ cho kế toán</t>
+    <t>Phát triển giao diện màn hình khởi tạo phân bổ cho kế toán</t>
   </si>
   <si>
-    <t xml:space="preserve">Giao diện chọn kỳ, nhập thông số và preview phân bổ.</t>
+    <t>Giao diện chọn kỳ, nhập thông số và preview phân bổ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cập nhật màn hình Quản lý giá vốn Cloudhub hiển thị hóa đơn trả trước</t>
+    <t>Cập nhật màn hình Quản lý giá vốn Cloudhub hiển thị hóa đơn trả trước</t>
   </si>
   <si>
-    <t xml:space="preserve">Bổ sung tab/filter phân loại trả tháng và trả trước.</t>
+    <t>Bổ sung tab/filter phân loại trả tháng và trả trước.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kế toán - Giá vốn &amp; Job</t>
+    <t>Kế toán - Giá vốn &amp; Job</t>
   </si>
   <si>
-    <t xml:space="preserve">Phát triển chức năng điều chỉnh thông tin phân bổ Giá vốn cho kế toán</t>
+    <t>Phát triển chức năng điều chỉnh thông tin phân bổ Giá vốn cho kế toán</t>
   </si>
   <si>
-    <t xml:space="preserve">Điều chỉnh giá vốn, lập Job khóa dữ liệu và Unit Test Kế toán.</t>
+    <t>Điều chỉnh giá vốn, lập Job khóa dữ liệu và Unit Test Kế toán.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sửa giá vốn import kèm lưu log audit trail lịch sử.</t>
+    <t>Sửa giá vốn import kèm lưu log audit trail lịch sử.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phát triển Background Job tự động khóa dữ liệu phân bổ theo kỳ lương</t>
+    <t>Phát triển Background Job tự động khóa dữ liệu phân bổ theo kỳ lương</t>
   </si>
   <si>
-    <t xml:space="preserve">Cron job khóa kỳ tự động, chặn sửa sau deadline.</t>
+    <t>Cron job khóa kỳ tự động, chặn sửa sau deadline.</t>
   </si>
   <si>
-    <t xml:space="preserve">Viết Unit Test chức năng phân bổ và giá vốn cho kế toán (AI-generated tests)</t>
+    <t>Viết Unit Test chức năng phân bổ và giá vốn cho kế toán (AI-generated tests)</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit test tự động cho hàm phân bổ và validate giá vốn.</t>
+    <t>Unit test tự động cho hàm phân bổ và validate giá vốn.</t>
   </si>
   <si>
-    <t xml:space="preserve">EPIC-2. Tích hợp hóa đơn Cloudhub và Danh mục FOXSG</t>
+    <t>EPIC-2. Tích hợp hóa đơn Cloudhub và Danh mục FOXSG</t>
   </si>
   <si>
-    <t xml:space="preserve">Tích hợp Billing Inside</t>
+    <t>Tích hợp Billing Inside</t>
   </si>
   <si>
-    <t xml:space="preserve">Xây dựng API Client &amp; Service tiếp nhận đồng bộ hóa đơn trả trước từ Inside</t>
+    <t>Xây dựng API Client &amp; Service tiếp nhận đồng bộ hóa đơn trả trước từ Inside</t>
   </si>
   <si>
-    <t xml:space="preserve">Tích hợp API đồng bộ hóa đơn Cloudhub từ Billing Inside về SAL.</t>
+    <t>Tích hợp API đồng bộ hóa đơn Cloudhub từ Billing Inside về SAL.</t>
   </si>
   <si>
-    <t xml:space="preserve">API auth token, retry mechanism khi timeout Inside.</t>
+    <t>API auth token, retry mechanism khi timeout Inside.</t>
   </si>
   <si>
-    <t xml:space="preserve">Xây dựng cơ chế Validate và lưu trữ hóa đơn Cloudhub trả trước vào SAL</t>
+    <t>Xây dựng cơ chế Validate và lưu trữ hóa đơn Cloudhub trả trước vào SAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Check trùng mã hóa đơn, mapping thời hạn và chu kỳ.</t>
+    <t>Check trùng mã hóa đơn, mapping thời hạn và chu kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Danh mục FOXSG</t>
+    <t>Danh mục FOXSG</t>
   </si>
   <si>
-    <t xml:space="preserve">Thiết kế Backend API quản lý danh mục hợp đồng FOXSG (AI boilerplate)</t>
+    <t>Thiết kế Backend API quản lý danh mục hợp đồng FOXSG (AI boilerplate)</t>
   </si>
   <si>
-    <t xml:space="preserve">Quản lý, tìm kiếm và đồng bộ danh mục hợp đồng FOXSG.</t>
+    <t>Quản lý, tìm kiếm và đồng bộ danh mục hợp đồng FOXSG.</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD danh mục FOXSG, tìm kiếm, lọc và phân quyền.</t>
+    <t>CRUD danh mục FOXSG, tìm kiếm, lọc và phân quyền.</t>
   </si>
   <si>
-    <t xml:space="preserve">Xây dựng UI quản lý và tìm kiếm danh mục hợp đồng FOXSG</t>
+    <t>Xây dựng UI quản lý và tìm kiếm danh mục hợp đồng FOXSG</t>
   </si>
   <si>
-    <t xml:space="preserve">Giao diện danh sách và form thêm/sửa hợp đồng FOXSG.</t>
+    <t>Giao diện danh sách và form thêm/sửa hợp đồng FOXSG.</t>
   </si>
   <si>
-    <t xml:space="preserve">EPIC-3. Nghiệp vụ phân tách hóa đơn và điều chỉnh lương TDV</t>
+    <t>EPIC-3. Nghiệp vụ phân tách hóa đơn và điều chỉnh lương TDV</t>
   </si>
   <si>
-    <t xml:space="preserve">TDV - Phân tách hóa đơn</t>
+    <t>TDV - Phân tách hóa đơn</t>
   </si>
   <si>
-    <t xml:space="preserve">Xây dựng API phân tách doanh thu &amp; giá vốn hóa đơn trả trước cho TDV</t>
+    <t>Xây dựng API phân tách doanh thu &amp; giá vốn hóa đơn trả trước cho TDV</t>
   </si>
   <si>
-    <t xml:space="preserve">Phân tách doanh thu/giá vốn hóa đơn trả trước cho TDV (UI &amp; Excel).</t>
+    <t>Phân tách doanh thu/giá vốn hóa đơn trả trước cho TDV (UI &amp; Excel).</t>
   </si>
   <si>
-    <t xml:space="preserve">Bóc tách doanh thu theo chu kỳ và tỷ lệ bán hàng.</t>
+    <t>Bóc tách doanh thu theo chu kỳ và tỷ lệ bán hàng.</t>
   </si>
   <si>
-    <t xml:space="preserve">Xây dựng UI popup/màn hình phân tách hóa đơn trả trước cho TDV</t>
+    <t>Xây dựng UI popup/màn hình phân tách hóa đơn trả trước cho TDV</t>
   </si>
   <si>
-    <t xml:space="preserve">Giao diện chia doanh số và giá vốn theo dòng cho TDV.</t>
+    <t>Giao diện chia doanh số và giá vốn theo dòng cho TDV.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phát triển chức năng Import Excel phân tách hóa đơn trả trước cho TDV</t>
+    <t>Phát triển chức năng Import Excel phân tách hóa đơn trả trước cho TDV</t>
   </si>
   <si>
-    <t xml:space="preserve">Template Excel, validate hàng loạt, báo lỗi từng dòng.</t>
+    <t>Template Excel, validate hàng loạt, báo lỗi từng dòng.</t>
   </si>
   <si>
-    <t xml:space="preserve">Điều chỉnh logic &amp; UI phân tách hóa đơn trả tháng cho TDV</t>
+    <t>Điều chỉnh logic &amp; UI phân tách hóa đơn trả tháng cho TDV</t>
   </si>
   <si>
-    <t xml:space="preserve">Đồng bộ giao diện và logic phân tách trả tháng/trả trước.</t>
+    <t>Đồng bộ giao diện và logic phân tách trả tháng/trả trước.</t>
   </si>
   <si>
-    <t xml:space="preserve">TDV - Điều chỉnh lương</t>
+    <t>TDV - Điều chỉnh lương</t>
   </si>
   <si>
-    <t xml:space="preserve">Phát triển tính năng load danh sách và cập nhật thông tin tính lương cho TDV</t>
+    <t>Phát triển tính năng load danh sách và cập nhật thông tin tính lương cho TDV</t>
   </si>
   <si>
-    <t xml:space="preserve">Điều chỉnh thông tin tính lương TDV và Unit Test phân hệ TDV.</t>
+    <t>Điều chỉnh thông tin tính lương TDV và Unit Test phân hệ TDV.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cho phép TDV/BOD chỉnh sửa trực tiếp thông số lương.</t>
+    <t>Cho phép TDV/BOD chỉnh sửa trực tiếp thông số lương.</t>
   </si>
   <si>
-    <t xml:space="preserve">Viết Unit Test chức năng phân bổ và điều chỉnh lương cho TDV (AI-generated)</t>
+    <t>Viết Unit Test chức năng phân bổ và điều chỉnh lương cho TDV (AI-generated)</t>
   </si>
   <si>
-    <t xml:space="preserve">EPIC-4. Bảng lương và Core tính lương hóa đơn Cloudhub</t>
+    <t>EPIC-4. Bảng lương và Core tính lương hóa đơn Cloudhub</t>
   </si>
   <si>
-    <t xml:space="preserve">Core lương - Logic tính toán</t>
+    <t>Core lương - Logic tính toán</t>
   </si>
   <si>
-    <t xml:space="preserve">Điều chỉnh Core lương hóa đơn trả tháng Cloudhub theo quy tắc mới</t>
+    <t>Điều chỉnh Core lương hóa đơn trả tháng Cloudhub theo quy tắc mới</t>
   </si>
   <si>
-    <t xml:space="preserve">Nâng cấp Core tính lương trả tháng và bổ sung giải thuật trả trước.</t>
+    <t>Nâng cấp Core tính lương trả tháng và bổ sung giải thuật trả trước.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tinh chỉnh điều kiện xét mốc và công thức trả tháng.</t>
+    <t>Tinh chỉnh điều kiện xét mốc và công thức trả tháng.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phát triển nhánh Core lương hóa đơn trả trước Cloudhub (bóc tách chu kỳ)</t>
+    <t>Phát triển nhánh Core lương hóa đơn trả trước Cloudhub (bóc tách chu kỳ)</t>
   </si>
   <si>
-    <t xml:space="preserve">Giải thuật bóc tách doanh thu theo chu kỳ &gt;12 tháng.</t>
+    <t>Giải thuật bóc tách doanh thu theo chu kỳ &gt;12 tháng.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bảng lương &amp; Export Excel</t>
+    <t>Bảng lương &amp; Export Excel</t>
   </si>
   <si>
-    <t xml:space="preserve">Xây dựng tab hiển thị và bảng lương hóa đơn trả trước Cloudhub</t>
+    <t>Xây dựng tab hiển thị và bảng lương hóa đơn trả trước Cloudhub</t>
   </si>
   <si>
-    <t xml:space="preserve">Bảng lương hóa đơn trả trước, xuất Excel và Unit Test Core lương.</t>
+    <t>Bảng lương hóa đơn trả trước, xuất Excel và Unit Test Core lương.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tab bảng lương sản phẩm riêng, hiển thị chi tiết cột tính.</t>
+    <t>Tab bảng lương sản phẩm riêng, hiển thị chi tiết cột tính.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phát triển tính năng xuất Excel bảng lương hóa đơn trả trước Cloudhub</t>
+    <t>Phát triển tính năng xuất Excel bảng lương hóa đơn trả trước Cloudhub</t>
   </si>
   <si>
-    <t xml:space="preserve">Template xuất Excel đối soát chuẩn format.</t>
+    <t>Template xuất Excel đối soát chuẩn format.</t>
   </si>
   <si>
-    <t xml:space="preserve">Viết Unit Test chức năng bảng lương và giải thuật Core lương</t>
+    <t>Viết Unit Test chức năng bảng lương và giải thuật Core lương</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit test kiểm tra công thức toán học và số liệu bảng lương.</t>
+    <t>Unit test kiểm tra công thức toán học và số liệu bảng lương.</t>
   </si>
   <si>
-    <t xml:space="preserve">EPIC-5. QC / UAT / Deploy Staging / Sprint Ceremonies</t>
+    <t>EPIC-5. QC / UAT / Deploy Staging / Sprint Ceremonies</t>
   </si>
   <si>
-    <t xml:space="preserve">QC Onboarding &amp; Test Planning</t>
+    <t>QC Onboarding &amp; Test Planning</t>
   </si>
   <si>
-    <t xml:space="preserve">Demo &amp; Clear nghiệp vụ Sprint 2 cho đội ngũ QC</t>
+    <t>Demo &amp; Clear nghiệp vụ Sprint 2 cho đội ngũ QC</t>
   </si>
   <si>
-    <t xml:space="preserve">Onboarding, demo nghiệp vụ và viết Testcase cho 19 hạng mục.</t>
+    <t>Onboarding, demo nghiệp vụ và viết Testcase cho 19 hạng mục.</t>
   </si>
   <si>
-    <t xml:space="preserve">BA giải đáp luồng bóc tách hóa đơn, phân bổ và phân tách.</t>
+    <t>BA giải đáp luồng bóc tách hóa đơn, phân bổ và phân tách.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nghiên cứu PRD &amp; Viết Testcase nhóm Kế toán AF và Tích hợp Inside (Phần 1)</t>
+    <t>Nghiên cứu PRD &amp; Viết Testcase nhóm Kế toán AF và Tích hợp Inside (Phần 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">HaTTT65</t>
+    <t>HaTTT65</t>
   </si>
   <si>
-    <t xml:space="preserve">Testcase phân bổ AF, giá vốn, job khóa kỳ, sync Inside, FOXSG.</t>
+    <t>Testcase phân bổ AF, giá vốn, job khóa kỳ, sync Inside, FOXSG.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nghiên cứu PRD &amp; Viết Testcase nhóm TDV và Core Bảng lương (Phần 1)</t>
+    <t>Nghiên cứu PRD &amp; Viết Testcase nhóm TDV và Core Bảng lương (Phần 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">AnhDC4</t>
+    <t>AnhDC4</t>
   </si>
   <si>
-    <t xml:space="preserve">Testcase phân tách TDV, import excel, core lương, export.</t>
+    <t>Testcase phân tách TDV, import excel, core lương, export.</t>
   </si>
   <si>
-    <t xml:space="preserve">Review chéo Testcase &amp; Tối ưu kịch bản Test tích hợp hệ thống</t>
+    <t>Review chéo Testcase &amp; Tối ưu kịch bản Test tích hợp hệ thống</t>
   </si>
   <si>
-    <t xml:space="preserve">Review chéo giữa 2 QC đảm bảo bao phủ edge cases.</t>
+    <t>Review chéo giữa 2 QC đảm bảo bao phủ edge cases.</t>
   </si>
   <si>
-    <t xml:space="preserve">Thiết lập môi trường Automation &amp; Kịch bản Test hiệu năng API</t>
+    <t>Thiết lập môi trường Automation &amp; Kịch bản Test hiệu năng API</t>
   </si>
   <si>
-    <t xml:space="preserve">Script test API Inside sync và import excel hàng loạt.</t>
+    <t>Script test API Inside sync và import excel hàng loạt.</t>
   </si>
   <si>
-    <t xml:space="preserve">Deployment Staging &amp; Testing Execution</t>
+    <t>Deployment Staging &amp; Testing Execution</t>
   </si>
   <si>
-    <t xml:space="preserve">Deploy bản build hoàn thiện Sprint 2 lên môi trường Staging</t>
+    <t>Deploy bản build hoàn thiện Sprint 2 lên môi trường Staging</t>
   </si>
   <si>
-    <t xml:space="preserve">Deploy Staging, thực hiện QC Testing và xử lý bug.</t>
+    <t>Deploy Staging, thực hiện QC Testing và xử lý bug.</t>
   </si>
   <si>
-    <t xml:space="preserve">Migration DB Staging, check kết nối Inside trước test.</t>
+    <t>Migration DB Staging, check kết nối Inside trước test.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hỗ trợ nghiệp vụ cho đội ngũ QC execute</t>
+    <t>Hỗ trợ nghiệp vụ cho đội ngũ QC execute</t>
   </si>
   <si>
-    <t xml:space="preserve">BA standby giải đáp nghiệp vụ và verify bug report.</t>
+    <t>BA standby giải đáp nghiệp vụ và verify bug report.</t>
   </si>
   <si>
-    <t xml:space="preserve">Thực hiện QC Testing Round 1 nhóm Kế toán AF &amp; Tích hợp Inside</t>
+    <t>Thực hiện QC Testing Round 1 nhóm Kế toán AF &amp; Tích hợp Inside</t>
   </si>
   <si>
-    <t xml:space="preserve">Kiểm thử phân bổ AF, job khóa kỳ, sync Inside và FOXSG.</t>
+    <t>Kiểm thử phân bổ AF, job khóa kỳ, sync Inside và FOXSG.</t>
   </si>
   <si>
-    <t xml:space="preserve">Thực hiện QC Testing Round 1 nhóm TDV &amp; Core Bảng lương</t>
+    <t>Thực hiện QC Testing Round 1 nhóm TDV &amp; Core Bảng lương</t>
   </si>
   <si>
-    <t xml:space="preserve">Kiểm thử phân tách TDV, import excel, tính và xuất lương.</t>
+    <t>Kiểm thử phân tách TDV, import excel, tính và xuất lương.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix bug phát sinh từ QC Testing Round 1 (Phần 1)</t>
+    <t>Fix bug phát sinh từ QC Testing Round 1 (Phần 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix bug Critical/High phân hệ Kế toán AF và Inside.</t>
+    <t>Fix bug Critical/High phân hệ Kế toán AF và Inside.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix bug phát sinh từ QC Testing Round 1 (Phần 2)</t>
+    <t>Fix bug phát sinh từ QC Testing Round 1 (Phần 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix bug phân hệ TDV, Core lương và export Excel.</t>
+    <t>Fix bug phân hệ TDV, Core lương và export Excel.</t>
   </si>
   <si>
-    <t xml:space="preserve">Recheck bug đã fix &amp; Regression test phân hệ Kế toán và Tích hợp</t>
+    <t>Recheck bug đã fix &amp; Regression test phân hệ Kế toán và Tích hợp</t>
   </si>
   <si>
-    <t xml:space="preserve">Recheck bug đã fix, kiểm tra không lỗi chéo màn hình cũ.</t>
+    <t>Recheck bug đã fix, kiểm tra không lỗi chéo màn hình cũ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Recheck bug đã fix &amp; Regression test phân hệ TDV và Bảng lương</t>
+    <t>Recheck bug đã fix &amp; Regression test phân hệ TDV và Bảng lương</t>
   </si>
   <si>
-    <t xml:space="preserve">Recheck bug Core lương, kiểm tra đối soát số liệu export.</t>
+    <t>Recheck bug Core lương, kiểm tra đối soát số liệu export.</t>
   </si>
   <si>
-    <t xml:space="preserve">UAT &amp; User Documentation</t>
+    <t>UAT &amp; User Documentation</t>
   </si>
   <si>
-    <t xml:space="preserve">Viết UAT, User Guide Scenario cho toàn bộ tính năng</t>
+    <t>Viết UAT, User Guide Scenario cho toàn bộ tính năng</t>
   </si>
   <si>
-    <t xml:space="preserve">Viết kịch bản UAT, User Guide và hỗ trợ người dùng nghiệm thu.</t>
+    <t>Viết kịch bản UAT, User Guide và hỗ trợ người dùng nghiệm thu.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kịch bản nghiệm thu chi tiết cho Kế toán AF và TDV.</t>
+    <t>Kịch bản nghiệm thu chi tiết cho Kế toán AF và TDV.</t>
   </si>
   <si>
-    <t xml:space="preserve">Viết User Guide hướng dẫn sử dụng tính năng mới</t>
+    <t>Viết User Guide hướng dẫn sử dụng tính năng mới</t>
   </si>
   <si>
-    <t xml:space="preserve">Tài liệu hướng dẫn kèm hình ảnh minh họa tính năng mới.</t>
+    <t>Tài liệu hướng dẫn kèm hình ảnh minh họa tính năng mới.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hướng dẫn và hỗ trợ người dùng thực hiện UAT</t>
+    <t>Hướng dẫn và hỗ trợ người dùng thực hiện UAT</t>
   </si>
   <si>
-    <t xml:space="preserve">Hỗ trợ Kế toán và TDV thao tác trực tiếp trên Staging.</t>
+    <t>Hỗ trợ Kế toán và TDV thao tác trực tiếp trên Staging.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix bug và hỗ trợ kỹ thuật trong quá trình UAT</t>
+    <t>Fix bug và hỗ trợ kỹ thuật trong quá trình UAT</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotfix ngay các vấn đề phát sinh trong buổi nghiệm thu.</t>
+    <t>Hotfix ngay các vấn đề phát sinh trong buổi nghiệm thu.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tổng hợp kết quả UAT và lấy UAT Sign-off chính thức</t>
+    <t>Tổng hợp kết quả UAT và lấy UAT Sign-off chính thức</t>
   </si>
   <si>
-    <t xml:space="preserve">Ký biên bản nghiệm thu UAT với Kế toán và TDV.</t>
+    <t>Ký biên bản nghiệm thu UAT với Kế toán và TDV.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint Ceremonies &amp; Release Management</t>
+    <t>Sprint Ceremonies &amp; Release Management</t>
   </si>
   <si>
-    <t xml:space="preserve">Tổ chức Sprint Review &amp; Báo cáo kết quả Sprint 2 cho Stakeholders</t>
+    <t>Tổ chức Sprint Review &amp; Báo cáo kết quả Sprint 2 cho Stakeholders</t>
   </si>
   <si>
-    <t xml:space="preserve">Đóng gói release Staging, tổ chức Sprint Review và Retrospective.</t>
+    <t>Đóng gói release Staging, tổ chức Sprint Review và Retrospective.</t>
   </si>
   <si>
-    <t xml:space="preserve">Demo tính năng hoàn thành, báo cáo chỉ số tiến độ/chất lượng.</t>
+    <t>Demo tính năng hoàn thành, báo cáo chỉ số tiến độ/chất lượng.</t>
   </si>
   <si>
-    <t xml:space="preserve">Đóng gói mã nguồn bản build Staging &amp; Bàn giao tài liệu kỹ thuật</t>
+    <t>Đóng gói mã nguồn bản build Staging &amp; Bàn giao tài liệu kỹ thuật</t>
   </si>
   <si>
-    <t xml:space="preserve">Đóng gói release package, tag git v3.1-sprint2 trên Staging.</t>
+    <t>Đóng gói release package, tag git v3.1-sprint2 trên Staging.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tổ chức Sprint Retrospective &amp; Hoàn tất đóng Sprint 2</t>
+    <t>Tổ chức Sprint Retrospective &amp; Hoàn tất đóng Sprint 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Họp rút kinh nghiệm, ghi nhận bài học và đóng Sprint trên Jira.</t>
+    <t>Họp rút kinh nghiệm, ghi nhận bài học và đóng Sprint trên Jira.</t>
   </si>
   <si>
-    <t xml:space="preserve">Timeline &amp; Milestones</t>
+    <t>Timeline &amp; Milestones</t>
   </si>
   <si>
-    <t xml:space="preserve">UAT</t>
+    <t>UAT</t>
   </si>
   <si>
-    <t xml:space="preserve">PO tiến hành UAT</t>
+    <t>PO tiến hành UAT</t>
   </si>
   <si>
-    <t xml:space="preserve">PO</t>
+    <t>PO</t>
   </si>
   <si>
-    <t xml:space="preserve">0%</t>
+    <t>0%</t>
   </si>
   <si>
-    <t xml:space="preserve">ORG CHART &amp; COMMUNICATION PLAN</t>
+    <t>ORG CHART &amp; COMMUNICATION PLAN</t>
   </si>
   <si>
-    <t xml:space="preserve">I. ORG CHART</t>
+    <t>I. ORG CHART</t>
   </si>
   <si>
-    <t xml:space="preserve">PROJECT TEAM</t>
+    <t>PROJECT TEAM</t>
   </si>
   <si>
-    <t xml:space="preserve">NO.</t>
+    <t>NO.</t>
   </si>
   <si>
-    <t xml:space="preserve">ACCOUNT EMAIL</t>
+    <t>ACCOUNT EMAIL</t>
   </si>
   <si>
-    <t xml:space="preserve">DIVISION</t>
+    <t>DIVISION</t>
   </si>
   <si>
-    <t xml:space="preserve">ROLE</t>
+    <t>ROLE</t>
   </si>
   <si>
-    <t xml:space="preserve">RESPONSIBILITY</t>
+    <t>RESPONSIBILITY</t>
   </si>
   <si>
-    <t xml:space="preserve">NhanNT3</t>
+    <t>NhanNT3</t>
   </si>
   <si>
-    <t xml:space="preserve">ISC</t>
+    <t>ISC</t>
   </si>
   <si>
-    <t xml:space="preserve">BGĐ ISC</t>
+    <t>BGĐ ISC</t>
   </si>
   <si>
-    <t xml:space="preserve">ThuyHK2</t>
+    <t>ThuyHK2</t>
   </si>
   <si>
-    <t xml:space="preserve">PMO</t>
+    <t>PMO</t>
   </si>
   <si>
-    <t xml:space="preserve">Project Management Operator – Quản lý PM, phân bổ nguồn lực cho dự án, đánh giá, đưa ra các giải pháp phù hợp.</t>
+    <t>Project Management Operator – Quản lý PM, phân bổ nguồn lực cho dự án, đánh giá, đưa ra các giải pháp phù hợp.</t>
   </si>
   <si>
-    <t xml:space="preserve">PM</t>
+    <t>PM</t>
   </si>
   <si>
-    <t xml:space="preserve">Quản trị dự án</t>
+    <t>Quản trị dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">ThaoTTT48</t>
+    <t>ThaoTTT48</t>
   </si>
   <si>
-    <t xml:space="preserve">QA</t>
+    <t>QA</t>
   </si>
   <si>
-    <t xml:space="preserve">Cán bộ đảm bảo chất lượng phần mềm</t>
+    <t>Cán bộ đảm bảo chất lượng phần mềm</t>
   </si>
   <si>
-    <t xml:space="preserve">OanhNTK35</t>
+    <t>OanhNTK35</t>
   </si>
   <si>
-    <t xml:space="preserve">BA</t>
+    <t>BA</t>
   </si>
   <si>
-    <t xml:space="preserve">Cán bộ phân tích nghiệp vụ</t>
+    <t>Cán bộ phân tích nghiệp vụ</t>
   </si>
   <si>
-    <t xml:space="preserve">PTL</t>
+    <t>PTL</t>
   </si>
   <si>
-    <t xml:space="preserve">Phụ trách các công việc liên quan đến kỹ thuật dự án.</t>
+    <t>Phụ trách các công việc liên quan đến kỹ thuật dự án.</t>
   </si>
   <si>
-    <t xml:space="preserve">QC</t>
+    <t>QC</t>
   </si>
   <si>
-    <t xml:space="preserve">Cán bộ kiểm thử phần mềm</t>
+    <t>Cán bộ kiểm thử phần mềm</t>
   </si>
   <si>
-    <t xml:space="preserve">DanhDC4</t>
+    <t>DanhDC4</t>
   </si>
   <si>
-    <t xml:space="preserve">DBA</t>
+    <t>DBA</t>
   </si>
   <si>
-    <t xml:space="preserve">Cán bộ quản trị database</t>
+    <t>Cán bộ quản trị database</t>
   </si>
   <si>
-    <t xml:space="preserve">Stakeholders</t>
+    <t>Stakeholders</t>
   </si>
   <si>
-    <t xml:space="preserve">LinhNVV2</t>
+    <t>LinhNVV2</t>
   </si>
   <si>
-    <t xml:space="preserve">FHR</t>
+    <t>FHR</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng hợp yêu cầu của EU 
@@ -888,75 +867,75 @@
 Push PO confirm URD , UAT đúng deadline</t>
   </si>
   <si>
-    <t xml:space="preserve">NhungVT2</t>
+    <t>NhungVT2</t>
   </si>
   <si>
-    <t xml:space="preserve">HR</t>
+    <t>HR</t>
   </si>
   <si>
-    <t xml:space="preserve">BO</t>
+    <t>BO</t>
   </si>
   <si>
-    <t xml:space="preserve">Cung cấp nghiệp vụ cho dự án</t>
+    <t>Cung cấp nghiệp vụ cho dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">NghiaDN</t>
+    <t>NghiaDN</t>
   </si>
   <si>
-    <t xml:space="preserve">Stakeholder</t>
+    <t>Stakeholder</t>
   </si>
   <si>
-    <t xml:space="preserve">Đảm bảo, xác nhận các yêu cầu và chất lượng phần mềm đã được đáp ứng</t>
+    <t>Đảm bảo, xác nhận các yêu cầu và chất lượng phần mềm đã được đáp ứng</t>
   </si>
   <si>
-    <t xml:space="preserve">Tranglth52</t>
+    <t>Tranglth52</t>
   </si>
   <si>
-    <t xml:space="preserve">FTIQA</t>
+    <t>FTIQA</t>
   </si>
   <si>
     <t xml:space="preserve">Hỗ trợ Quy trình của các chức năng , kiểm tra URD , 
 Tham gia UAT Test ,Pilot</t>
   </si>
   <si>
-    <t xml:space="preserve">Hangbt13</t>
+    <t>Hangbt13</t>
   </si>
   <si>
     <t xml:space="preserve">Đào tạo, hướng dẫn, cung cấp đầy đủthông tin vềquy trình, quy định trong quá trình thực hiện sốhóatại FTI
 Phối hợp và hỗtrợPD/POtrong việc giám sát, kiểm soát các hoạt động từphía FTI nhằm đảm bảo chất lượng dựán </t>
   </si>
   <si>
-    <t xml:space="preserve">VietNT8</t>
+    <t>VietNT8</t>
   </si>
   <si>
-    <t xml:space="preserve">ITSM</t>
+    <t>ITSM</t>
   </si>
   <si>
-    <t xml:space="preserve">HoangPV31</t>
+    <t>HoangPV31</t>
   </si>
   <si>
-    <t xml:space="preserve">AnhTT143</t>
+    <t>AnhTT143</t>
   </si>
   <si>
-    <t xml:space="preserve">GB</t>
+    <t>GB</t>
   </si>
   <si>
-    <t xml:space="preserve">HuyND6</t>
+    <t>HuyND6</t>
   </si>
   <si>
-    <t xml:space="preserve">Kĩ thuật</t>
+    <t>Kĩ thuật</t>
   </si>
   <si>
-    <t xml:space="preserve">TuDN</t>
+    <t>TuDN</t>
   </si>
   <si>
-    <t xml:space="preserve">VuPNK</t>
+    <t>VuPNK</t>
   </si>
   <si>
-    <t xml:space="preserve">FTI.ISC</t>
+    <t>FTI.ISC</t>
   </si>
   <si>
-    <t xml:space="preserve">PD</t>
+    <t>PD</t>
   </si>
   <si>
     <t xml:space="preserve">Nhiệm vụtrong quá trình thực hiện dựán sốhóa:
@@ -967,289 +946,289 @@
 ▪Xác định PO dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">HungNT50</t>
+    <t>HungNT50</t>
   </si>
   <si>
-    <t xml:space="preserve">CSOC</t>
+    <t>CSOC</t>
   </si>
   <si>
-    <t xml:space="preserve">Hỗ trợ phân bổ nguồn lực pentest dự án</t>
+    <t>Hỗ trợ phân bổ nguồn lực pentest dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">SonVH13</t>
+    <t>SonVH13</t>
   </si>
   <si>
-    <t xml:space="preserve">FTI SYSTEM</t>
+    <t>FTI SYSTEM</t>
   </si>
   <si>
-    <t xml:space="preserve">SYS</t>
+    <t>SYS</t>
   </si>
   <si>
-    <t xml:space="preserve">Cán bộ quản trị hệ thống git, cicd</t>
+    <t>Cán bộ quản trị hệ thống git, cicd</t>
   </si>
   <si>
-    <t xml:space="preserve">II. COMMUNICATION PLAN</t>
+    <t>II. COMMUNICATION PLAN</t>
   </si>
   <si>
-    <t xml:space="preserve">[Kế hoạch giao tiếp giữa PO, Stakeholder và Team dự án nhằm quản lý chặt chẽ yêu cầu, tiến độ dự án, quản lý issue và có action xử lý kịp thời.]</t>
+    <t>[Kế hoạch giao tiếp giữa PO, Stakeholder và Team dự án nhằm quản lý chặt chẽ yêu cầu, tiến độ dự án, quản lý issue và có action xử lý kịp thời.]</t>
   </si>
   <si>
-    <t xml:space="preserve">COMMUNICATION PLAN</t>
+    <t>COMMUNICATION PLAN</t>
   </si>
   <si>
-    <t xml:space="preserve">METHOD</t>
+    <t>METHOD</t>
   </si>
   <si>
-    <t xml:space="preserve">PARTICIPANTS</t>
+    <t>PARTICIPANTS</t>
   </si>
   <si>
-    <t xml:space="preserve">WHEN</t>
+    <t>WHEN</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm với PO v/v URD, PP, UAT, Change Request &amp; Release note</t>
+    <t>Confirm với PO v/v URD, PP, UAT, Change Request &amp; Release note</t>
   </si>
   <si>
-    <t xml:space="preserve">Email, MS Teams, Meeting minutes</t>
+    <t>Email, MS Teams, Meeting minutes</t>
   </si>
   <si>
-    <t xml:space="preserve">PO, Stakeholder và Group mail Team dự án</t>
+    <t>PO, Stakeholder và Group mail Team dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">By event</t>
+    <t>By event</t>
   </si>
   <si>
-    <t xml:space="preserve">Trao đổi, review tài liệu giữa PO, Stakeholder và Team dự án</t>
+    <t>Trao đổi, review tài liệu giữa PO, Stakeholder và Team dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">MS Teams</t>
+    <t>MS Teams</t>
   </si>
   <si>
-    <t xml:space="preserve">PO, Stakeholder và Group chat Team dự án</t>
+    <t>PO, Stakeholder và Group chat Team dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">Họp hàng tuần với PO</t>
+    <t>Họp hàng tuần với PO</t>
   </si>
   <si>
-    <t xml:space="preserve">Conference, MS Teams, face to face…</t>
+    <t>Conference, MS Teams, face to face…</t>
   </si>
   <si>
-    <t xml:space="preserve">PO, Stakeholder và Team dự án</t>
+    <t>PO, Stakeholder và Team dự án</t>
   </si>
   <si>
-    <t xml:space="preserve">Weekly</t>
+    <t>Weekly</t>
   </si>
   <si>
-    <t xml:space="preserve">Gửi báo cáo tuần cho PO</t>
+    <t>Gửi báo cáo tuần cho PO</t>
   </si>
   <si>
-    <t xml:space="preserve">Email</t>
+    <t>Email</t>
   </si>
   <si>
-    <t xml:space="preserve">PROJECT OBJECTIVES</t>
+    <t>PROJECT OBJECTIVES</t>
   </si>
   <si>
-    <t xml:space="preserve">Goals</t>
+    <t>Goals</t>
   </si>
   <si>
-    <t xml:space="preserve">Metrics</t>
+    <t>Metrics</t>
   </si>
   <si>
-    <t xml:space="preserve">UNIT</t>
+    <t>UNIT</t>
   </si>
   <si>
-    <t xml:space="preserve">Plan</t>
+    <t>Plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Priority</t>
+    <t>Priority</t>
   </si>
   <si>
-    <t xml:space="preserve">Rationale for target</t>
+    <t>Rationale for target</t>
   </si>
   <si>
-    <t xml:space="preserve">Condition/Constrains/ Risk</t>
+    <t>Condition/Constrains/ Risk</t>
   </si>
   <si>
-    <t xml:space="preserve">Min</t>
+    <t>Min</t>
   </si>
   <si>
-    <t xml:space="preserve">Max</t>
+    <t>Max</t>
   </si>
   <si>
-    <t xml:space="preserve">Follow process standard</t>
+    <t>Follow process standard</t>
   </si>
   <si>
-    <t xml:space="preserve">PCV</t>
+    <t>PCV</t>
   </si>
   <si>
-    <t xml:space="preserve">Point</t>
+    <t>Point</t>
   </si>
   <si>
-    <t xml:space="preserve">High</t>
+    <t>High</t>
   </si>
   <si>
-    <t xml:space="preserve">Based on ISC target</t>
+    <t>Based on ISC target</t>
   </si>
   <si>
-    <t xml:space="preserve">Need support from SQA actively and frequently.</t>
+    <t>Need support from SQA actively and frequently.</t>
   </si>
   <si>
-    <t xml:space="preserve">Improve customer satisfaction</t>
+    <t>Improve customer satisfaction</t>
   </si>
   <si>
-    <t xml:space="preserve">CSAT</t>
+    <t>CSAT</t>
   </si>
   <si>
-    <t xml:space="preserve">Customer</t>
+    <t>Customer</t>
   </si>
   <si>
-    <t xml:space="preserve">Customer usually requires higher quality</t>
+    <t>Customer usually requires higher quality</t>
   </si>
   <si>
-    <t xml:space="preserve">Keep plan of duration (Time)</t>
+    <t>Keep plan of duration (Time)</t>
   </si>
   <si>
-    <t xml:space="preserve">SPI (Schedule performance Index)</t>
+    <t>SPI (Schedule performance Index)</t>
   </si>
   <si>
-    <t xml:space="preserve">Buffer 10% for over estimation</t>
+    <t>Buffer 10% for over estimation</t>
   </si>
   <si>
-    <t xml:space="preserve">Requirement is not changed</t>
+    <t>Requirement is not changed</t>
   </si>
   <si>
-    <t xml:space="preserve">Keep plan of cost (Effort)</t>
+    <t>Keep plan of cost (Effort)</t>
   </si>
   <si>
-    <t xml:space="preserve">CPI (Cost performance Index)</t>
+    <t>CPI (Cost performance Index)</t>
   </si>
   <si>
     <t xml:space="preserve">
 Base on history data </t>
   </si>
   <si>
-    <t xml:space="preserve">RISK MANAGEMENT</t>
+    <t>RISK MANAGEMENT</t>
   </si>
   <si>
-    <t xml:space="preserve">Risk Priority</t>
+    <t>Risk Priority</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Score</t>
+    <t>Total Score</t>
   </si>
   <si>
     <t xml:space="preserve">Risk Response
 </t>
   </si>
   <si>
-    <t xml:space="preserve">6, 9</t>
+    <t>6, 9</t>
   </si>
   <si>
-    <t xml:space="preserve">Advoid, Transfer, Reduce</t>
+    <t>Advoid, Transfer, Reduce</t>
   </si>
   <si>
-    <t xml:space="preserve">Medium</t>
+    <t>Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">2, 3, 4</t>
+    <t>2, 3, 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Reduce, Transfer</t>
+    <t>Reduce, Transfer</t>
   </si>
   <si>
-    <t xml:space="preserve">Low</t>
+    <t>Low</t>
   </si>
   <si>
-    <t xml:space="preserve">Accept</t>
+    <t>Accept</t>
   </si>
   <si>
     <t xml:space="preserve"> [Dưới đây là ví dụ tham khảo, team dự án có thể customize lại &amp; log lên hệ thống để quản lý]</t>
   </si>
   <si>
-    <t xml:space="preserve">No.</t>
+    <t>No.</t>
   </si>
   <si>
-    <t xml:space="preserve">Risk type</t>
+    <t>Risk type</t>
   </si>
   <si>
-    <t xml:space="preserve">Action</t>
+    <t>Action</t>
   </si>
   <si>
-    <t xml:space="preserve">Probability</t>
+    <t>Probability</t>
   </si>
   <si>
-    <t xml:space="preserve">Impact</t>
+    <t>Impact</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL SCORE
 =LS * IS</t>
   </si>
   <si>
-    <t xml:space="preserve">Scope</t>
+    <t>Scope</t>
   </si>
   <si>
-    <t xml:space="preserve">**Change requests and project scope** – Phát sinh yêu cầu thay đổi/bổ sung scope, ảnh hưởng effort và kế hoạch.</t>
+    <t>**Change requests and project scope** – Phát sinh yêu cầu thay đổi/bổ sung scope, ảnh hưởng effort và kế hoạch.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phân tích, đánh giá impact; nếu phát sinh ≥10% effort thì tổ chức meeting và re-plan.</t>
+    <t>Phân tích, đánh giá impact; nếu phát sinh ≥10% effort thì tổ chức meeting và re-plan.</t>
   </si>
   <si>
-    <t xml:space="preserve">2-Medium</t>
+    <t>2-Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">3-High</t>
+    <t>3-High</t>
   </si>
   <si>
-    <t xml:space="preserve">Schedule</t>
+    <t>Schedule</t>
   </si>
   <si>
-    <t xml:space="preserve">**UAT and Pilot timelines cannot be guaranteed** – Timeline UAT/Pilot có thể bị ảnh hưởng do issue hoặc cần thêm thời gian phát triển.</t>
+    <t>**UAT and Pilot timelines cannot be guaranteed** – Timeline UAT/Pilot có thể bị ảnh hưởng do issue hoặc cần thêm thời gian phát triển.</t>
   </si>
   <si>
-    <t xml:space="preserve">Chủ động hỗ trợ EU, follow-up tiến độ; nếu cần thêm thời gian thì PO xác nhận và re-plan.</t>
+    <t>Chủ động hỗ trợ EU, follow-up tiến độ; nếu cần thêm thời gian thì PO xác nhận và re-plan.</t>
   </si>
   <si>
-    <t xml:space="preserve">Requirement</t>
+    <t>Requirement</t>
   </si>
   <si>
-    <t xml:space="preserve">**Does not yet meet EU requirements** – Chưa đáp ứng đầy đủ yêu cầu thực tế từ EU, đặc biệt các nghiệp vụ GB/OCC.</t>
+    <t>**Does not yet meet EU requirements** – Chưa đáp ứng đầy đủ yêu cầu thực tế từ EU, đặc biệt các nghiệp vụ GB/OCC.</t>
   </si>
   <si>
-    <t xml:space="preserve">Thu thập và xác nhận yêu cầu từ End-user (HR, Tech, Sales), ưu tiên GB/OCC.</t>
+    <t>Thu thập và xác nhận yêu cầu từ End-user (HR, Tech, Sales), ưu tiên GB/OCC.</t>
   </si>
   <si>
-    <t xml:space="preserve">Resource</t>
+    <t>Resource</t>
   </si>
   <si>
-    <t xml:space="preserve">**Shared resources for development and operations** – Resource dùng chung cho phát triển và vận hành, có thể ảnh hưởng capacity.</t>
+    <t>**Shared resources for development and operations** – Resource dùng chung cho phát triển và vận hành, có thể ảnh hưởng capacity.</t>
   </si>
   <si>
-    <t xml:space="preserve">Backup thêm effort vận hành song song với phát triển tính năng mới.</t>
+    <t>Backup thêm effort vận hành song song với phát triển tính năng mới.</t>
   </si>
   <si>
-    <t xml:space="preserve">REVISION HISTORY - PROJECT</t>
+    <t>REVISION HISTORY - PROJECT</t>
   </si>
   <si>
-    <t xml:space="preserve">Date</t>
+    <t>Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Version</t>
+    <t>Version</t>
   </si>
   <si>
-    <t xml:space="preserve">Author</t>
+    <t>Author</t>
   </si>
   <si>
-    <t xml:space="preserve">Reviewer</t>
+    <t>Reviewer</t>
   </si>
   <si>
-    <t xml:space="preserve">Approver</t>
+    <t>Approver</t>
   </si>
   <si>
-    <t xml:space="preserve">Change Description</t>
+    <t>Change Description</t>
   </si>
   <si>
-    <t xml:space="preserve">v3.7.1</t>
+    <t>v3.7.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Tạo mới</t>
+    <t>Tạo mới</t>
   </si>
 </sst>
 </file>
@@ -3115,7 +3094,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -10098,7 +10077,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="false"/>
@@ -19489,7 +19468,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="false"/>
@@ -22420,7 +22399,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -26066,7 +26045,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -27334,7 +27313,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -34774,7 +34753,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>

</xml_diff>